<commit_message>
Update app with payment flow, barcode, OCR, UI changes
</commit_message>
<xml_diff>
--- a/Face_Attendance/Attendance/Attendance_Log.xlsx
+++ b/Face_Attendance/Attendance/Attendance_Log.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,33 +465,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>akshay</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-01-29</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>18:50:51</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>